<commit_message>
Update Invenio records (2026-01-21)
</commit_message>
<xml_diff>
--- a/data/2026-01-21_invenio-records.xlsx
+++ b/data/2026-01-21_invenio-records.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
separate authors by "and"
</commit_message>
<xml_diff>
--- a/data/2026-01-21_invenio-records.xlsx
+++ b/data/2026-01-21_invenio-records.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -493,7 +493,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Ott, Caroline, Sommer, Frederik</t>
+          <t>Ott, Caroline and Sommer, Frederik</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -530,7 +530,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Kröninger, Lena, Maurya, Anay Kumar, Stiebeling, Christian, Stirba, Florian, Kim, Zio, Nowack, Eva</t>
+          <t>Kröninger, Lena and Maurya, Anay Kumar and Stiebeling, Christian and Stirba, Florian and Kim, Zio and Nowack, Eva</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -567,7 +567,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Krüger, Aileen, Göddecke, Janik, Osthege, Michael, Navratil, Luis, Weber, Ulrike, Oldiges, Marco, Frunzke, Julia</t>
+          <t>Krüger, Aileen and Göddecke, Janik and Osthege, Michael and Navratil, Luis and Weber, Ulrike and Oldiges, Marco and Frunzke, Julia</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -604,7 +604,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Feldbrügge, Michael, Müntjes, Kira, Mann, Marcel, Richter, Paul, Philipp, Magnus, Plücker, Lesley, Schipper, Kerstin</t>
+          <t>Feldbrügge, Michael and Müntjes, Kira and Mann, Marcel and Richter, Paul and Philipp, Magnus and Plücker, Lesley and Schipper, Kerstin</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Zöllner, Nora R., Sharkey, Jacob E., Frommer, Wolf B.</t>
+          <t>Zöllner, Nora R. and Sharkey, Jacob E. and Frommer, Wolf B.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Papadopoulos, Athanasios, Anlauf, Manuel, Reiners, Jens, Paik, Sueng-Hyun, Krueger, Aileen, Lueckel, Benita, Bott, Michael, Drepper, Thomas, Frunzke, Julia, Gohlke, Holger, Weidtkamp-Peters, Stefanie, Smits, Sander, Gertzen, Christoph</t>
+          <t>Papadopoulos, Athanasios and Anlauf, Manuel and Reiners, Jens and Paik, Sueng-Hyun and Krueger, Aileen and Lueckel, Benita and Bott, Michael and Drepper, Thomas and Frunzke, Julia and Gohlke, Holger and Weidtkamp-Peters, Stefanie and Smits, Sander and Gertzen, Christoph</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Krüger, Aileen, Frunzke, Julia, Weber, Ulrike</t>
+          <t>Krüger, Aileen and Frunzke, Julia and Weber, Ulrike</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -752,7 +752,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Helmsorig, Gesa, Lan, Tianyu, Haraldsson, Einar Baldvin, Rütjes, Thea, Westhoff, Philipp, Weber, Katrin, Kumlehn, Jochen, Hensel, Götz, Simon, Rüdiger, von Korff, Maria</t>
+          <t>Helmsorig, Gesa and Lan, Tianyu and Haraldsson, Einar Baldvin and Rütjes, Thea and Westhoff, Philipp and Weber, Katrin and Kumlehn, Jochen and Hensel, Götz and Simon, Rüdiger and von Korff, Maria</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Ishikawa, Yuuma, Zöllner, Nora R., Paradies, Suanne, Frommer, Wolf B.</t>
+          <t>Ishikawa, Yuuma and Zöllner, Nora R. and Paradies, Suanne and Frommer, Wolf B.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -826,7 +826,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Rensing, Stefan, de Vries, Jan, Varshney, Deepti, Hiltemann, Saskia</t>
+          <t>Rensing, Stefan and de Vries, Jan and Varshney, Deepti and Hiltemann, Saskia</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -863,7 +863,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Dörpholz, Hannah, Demesa-Arevalo, Edgar, Usadel, Björn, Simon, Rüdiger</t>
+          <t>Dörpholz, Hannah and Demesa-Arevalo, Edgar and Usadel, Björn and Simon, Rüdiger</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Zappone, Dario, Schwechheimer, Claus, Schröder, Peter Michael, Kerstin Becker, Schneeberger, Korbinian, Dong, Xiao, Novák, Ondřej, Ivan Petřík, Rudolf  Schäufele</t>
+          <t>Zappone, Dario and Schwechheimer, Claus and Schröder, Peter Michael and Kerstin Becker and Schneeberger, Korbinian and Dong, Xiao and Novák, Ondřej and Ivan Petřík and Rudolf  Schäufele</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Kaplunova, Vera, Alioui, Houda, Griguschies, Tobias, Durán, Paloma, Lautwein, Tobias, Metzger, Sabine, Loo, Eliza</t>
+          <t>Kaplunova, Vera and Alioui, Houda and Griguschies, Tobias and Durán, Paloma and Lautwein, Tobias and Metzger, Sabine and Loo, Eliza</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Annunziata, Maria Grazia, Feil, Regina, Lohse, Marc, Figueroa, Carlos, Hartman, Matías, Esmailpour, Mohammad, Nikoloski, Zoran, Koehl, Karin, Stitt, Mark, Lunn, John, Fichtner, Franziska</t>
+          <t>Annunziata, Maria Grazia and Feil, Regina and Lohse, Marc and Figueroa, Carlos and Hartman, Matías and Esmailpour, Mohammad and Nikoloski, Zoran and Koehl, Karin and Stitt, Mark and Lunn, John and Fichtner, Franziska</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Foth, Natalie, Fäßler, Moritz, Ott, Caroline, Muehlhaus, Timo, Sommer, Frederik, Schroda, Michael, Kins, Stefan</t>
+          <t>Foth, Natalie and Fäßler, Moritz and Ott, Caroline and Muehlhaus, Timo and Sommer, Frederik and Schroda, Michael and Kins, Stefan</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Genzel, Franziska, Wiese-Klinkenberg, Anika</t>
+          <t>Genzel, Franziska and Wiese-Klinkenberg, Anika</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1122,7 +1122,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Frommer, Wolf B., Redzich, Laura</t>
+          <t>Frommer, Wolf B. and Redzich, Laura</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1159,7 +1159,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Bueno da Silva, Marília, Genzel, Franziska, Wiese-Klinkenberg, Anika, Bredenbruch, Sandra, Grundler, Florian M. W., Schleker, A. Sylvia S.</t>
+          <t>Bueno da Silva, Marília and Genzel, Franziska and Wiese-Klinkenberg, Anika and Bredenbruch, Sandra and Grundler, Florian M. W. and Schleker, A. Sylvia S.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Loo, Eliza, Huguet-Tapia, José, Selvaraj, Michael Gomez, Stiebner, Melissa, Killing, Britta, Buchholzer, Marcel, Schepler-Luu, Van, Hartwig, Thomas, Rivera Gutiérrez, Sandra, Rast-Somssich, Madlen Ingeborg, Szurek, Boris, Tohme, Joe, Charraviaga, Paul, White, Frank, Yang, Bing, Frommer, Wolf B.</t>
+          <t>Loo, Eliza and Huguet-Tapia, José and Selvaraj, Michael Gomez and Stiebner, Melissa and Killing, Britta and Buchholzer, Marcel and Schepler-Luu, Van and Hartwig, Thomas and Rivera Gutiérrez, Sandra and Rast-Somssich, Madlen Ingeborg and Szurek, Boris and Tohme, Joe and Charraviaga, Paul and White, Frank and Yang, Bing and Frommer, Wolf B.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Dann, Marcel, Eunchul, Kim, Pohland, Anne-Christin, Sommer, Frederik</t>
+          <t>Dann, Marcel and Eunchul, Kim and Pohland, Anne-Christin and Sommer, Frederik</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Senger, Elisa, McCallum, Susan, Jorgenson, Linzi, Britten, Avril, McCallum, James, Osti, Loris, Giacomelli, Sara, Olbricht, Klaus, Wagner, Henning, Waurich, Veronika, Predieri, Stefano, Daniele, Giulia Maria, Lippi, Nico, Magli, Massimiliano, Mazzoni, Luca, Capocasa, Franco, Marcellini, Micol, Giovanetti, Giammarco, Pergolotti, Valeria, Raffaelli, Davide, Qaderi, Rohullah, Franceschini, Matteo, Mecozzi, Federica, Kafkas, Ebru, Zucchi, Paolo, Savini, Gianluca, Toldo, Stefania, Cattani, Sabrina, Ayvaz Sönmez, Duygu, Perez Santana, Carlos, Piston Piston, Fernando, Arenas Pizarro, Juan Manuel, Lopez Rodriguez, Daniel, Cobano Cardeñas, Paloma, Rodriguez Mora, Ana Maria, Refoyo, Antonio, Borrero, Celia, Avilés, Manuel, Sanz, Carlos, Graham, Julie, Miranda Enamorado, Luis, Martinez Ferri, Elsa, Ariza Fernández, María Teresa, Soria Navarro, Carmen, Medina Mínguez, Juan Jesús, Muñoz, Pilar, Roldan Guerra, Francisco Javier, Verma, Sujeet, Ruiz-Velázque, Mario, Torreblanca, Rocío, Oiza, Nicolás, Castillejo, Cristina, Sánchez-Sevilla, José F., Amaya, Iraida, Davik, Jahn, Haikonen, Tuuli, Öz, Ayşe Tülin, Kafkas, Salih, Özgoren, Burak, Attar, Şule Hilal, Yeşil, Betül, Mezzetti, Bruno</t>
+          <t>Senger, Elisa and McCallum, Susan and Jorgenson, Linzi and Britten, Avril and McCallum, James and Osti, Loris and Giacomelli, Sara and Olbricht, Klaus and Wagner, Henning and Waurich, Veronika and Predieri, Stefano and Daniele, Giulia Maria and Lippi, Nico and Magli, Massimiliano and Mazzoni, Luca and Capocasa, Franco and Marcellini, Micol and Giovanetti, Giammarco and Pergolotti, Valeria and Raffaelli, Davide and Qaderi, Rohullah and Franceschini, Matteo and Mecozzi, Federica and Kafkas, Ebru and Zucchi, Paolo and Savini, Gianluca and Toldo, Stefania and Cattani, Sabrina and Ayvaz Sönmez, Duygu and Perez Santana, Carlos and Piston Piston, Fernando and Arenas Pizarro, Juan Manuel and Lopez Rodriguez, Daniel and Cobano Cardeñas, Paloma and Rodriguez Mora, Ana Maria and Refoyo, Antonio and Borrero, Celia and Avilés, Manuel and Sanz, Carlos and Graham, Julie and Miranda Enamorado, Luis and Martinez Ferri, Elsa and Ariza Fernández, María Teresa and Soria Navarro, Carmen and Medina Mínguez, Juan Jesús and Muñoz, Pilar and Roldan Guerra, Francisco Javier and Verma, Sujeet and Ruiz-Velázque, Mario and Torreblanca, Rocío and Oiza, Nicolás and Castillejo, Cristina and Sánchez-Sevilla, José F. and Amaya, Iraida and Davik, Jahn and Haikonen, Tuuli and Öz, Ayşe Tülin and Kafkas, Salih and Özgoren, Burak and Attar, Şule Hilal and Yeşil, Betül and Mezzetti, Bruno</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Arra, Yugander, Frommer, Wolf B., Redzich, Laura</t>
+          <t>Arra, Yugander and Frommer, Wolf B. and Redzich, Laura</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1344,7 +1344,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Scheid, Josephine Leonie, Schneider, Kevin, Mühlhaus, Timo</t>
+          <t>Scheid, Josephine Leonie and Schneider, Kevin and Mühlhaus, Timo</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Witting, Lennart, Seiffarth, Johannes, Stute, Birgit, Schulze, Tim, Hofer, Jan Matthis, Nöh, Katharina, Eisenhut, Marion, Weber, Andreas P. M., von Lieres, Eric, Kohlheyer, Dietrich</t>
+          <t>Witting, Lennart and Seiffarth, Johannes and Stute, Birgit and Schulze, Tim and Hofer, Jan Matthis and Nöh, Katharina and Eisenhut, Marion and Weber, Andreas P. M. and von Lieres, Eric and Kohlheyer, Dietrich</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1455,7 +1455,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Lan, Tianyu, Walla, Agatha, Çolpan Karışan, Kumsal Ecem, Buchmann, Gabriele, Wewer, Vera, Metzger, Sabine, Vardanega, Isaia, Haraldsson, Einar Baldvin, Helmsorig, Gesa, Thirulogachandar, Venkatasubbu, Simon, Rüdiger, von Korff, Maria</t>
+          <t>Lan, Tianyu and Walla, Agatha and Çolpan Karışan, Kumsal Ecem and Buchmann, Gabriele and Wewer, Vera and Metzger, Sabine and Vardanega, Isaia and Haraldsson, Einar Baldvin and Helmsorig, Gesa and Thirulogachandar, Venkatasubbu and Simon, Rüdiger and von Korff, Maria</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Ziegler, Freya, Rosenthal, Vivien, Vallarino, José G., Genzel, Franziska, Spettmann, Sarah, Seliga, Łukasz, Keller-Przybyłkowicz, Sylwia, Munnes, Lucas, Sønsteby, Anita, Osorio, Sonia, Usadel, Björn</t>
+          <t>Ziegler, Freya and Rosenthal, Vivien and Vallarino, José G. and Genzel, Franziska and Spettmann, Sarah and Seliga, Łukasz and Keller-Przybyłkowicz, Sylwia and Munnes, Lucas and Sønsteby, Anita and Osorio, Sonia and Usadel, Björn</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Erika, Csicsely, Top, Oguz, Frank, Wolfgang</t>
+          <t>Erika, Csicsely and Top, Oguz and Frank, Wolfgang</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Schladt, Till Moritz, Miras, Manuel, Ejike, Jona Obinna, Pottier, Mathieu, Xi, Lin, Restrepo, Andrea, Nakamura, Masayoshi, Pütz, Niklas, Hänsch, Sebastian, Gao, Chen, Engelhorn, Julia, Dickmanns, Marcel, Davis, Gwendolyn, Dalal, Ahan, Gombos, Sven, Lange, Ronja, Simon, Rüdiger, Schulze, Waltraud, Frommer, Wolf B.</t>
+          <t>Schladt, Till Moritz and Miras, Manuel and Ejike, Jona Obinna and Pottier, Mathieu and Xi, Lin and Restrepo, Andrea and Nakamura, Masayoshi and Pütz, Niklas and Hänsch, Sebastian and Gao, Chen and Engelhorn, Julia and Dickmanns, Marcel and Davis, Gwendolyn and Dalal, Ahan and Gombos, Sven and Lange, Ronja and Simon, Rüdiger and Schulze, Waltraud and Frommer, Wolf B.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Wijesingha Ahchige, Micha, Fisher, Josef, Sokolowska, Ewelina, Lyall, Rafe, Illing, Nicola, Skirycz, Aleksandra, Zamir, Dani, Alseekh, Saleh, Fernie, Alisdair</t>
+          <t>Wijesingha Ahchige, Micha and Fisher, Josef and Sokolowska, Ewelina and Lyall, Rafe and Illing, Nicola and Skirycz, Aleksandra and Zamir, Dani and Alseekh, Saleh and Fernie, Alisdair</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1640,7 +1640,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Tariq, Arslan, Meng, Minghui, Jiang, Xiaohui, Bolger, Anthony, Beier, Sebastian, Buchmann, Jan, Fernie, Alisdair, Wen, Weiwei, Usadel, Björn</t>
+          <t>Tariq, Arslan and Meng, Minghui and Jiang, Xiaohui and Bolger, Anthony and Beier, Sebastian and Buchmann, Jan and Fernie, Alisdair and Wen, Weiwei and Usadel, Björn</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1677,7 +1677,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Hess, Wolfgang, Heß, Daniel, Holzhausen, Anja</t>
+          <t>Hess, Wolfgang and Heß, Daniel and Holzhausen, Anja</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Frohn, Stephanie, Schippers, Jos</t>
+          <t>Frohn, Stephanie and Schippers, Jos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Kreiss, Melanie, Haas, Fabian, Hansen, Maike, Rensing, Stefan, Hoecker, Ute</t>
+          <t>Kreiss, Melanie and Haas, Fabian and Hansen, Maike and Rensing, Stefan and Hoecker, Ute</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1788,7 +1788,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Zhang, Ningning, Mattoon, Erin, McHargue, Will, Venn, Benedikt, Zimmer, David, Pecani, Kresti, Jeong, Jooyeon, Anderson, Cheyenne, Chen, Chen, Berry, Jeffrey, Xia, Ming, Tzeng, Shin-Cheng, Becker, Eric, Pazouki, Leila, Evans, Bradley, Cross, Fred, Cheng, Jianlin, Czymmek, Kirk, Schroda, Michael, Mühlhaus, Timo, Zhang, Ru</t>
+          <t>Zhang, Ningning and Mattoon, Erin and McHargue, Will and Venn, Benedikt and Zimmer, David and Pecani, Kresti and Jeong, Jooyeon and Anderson, Cheyenne and Chen, Chen and Berry, Jeffrey and Xia, Ming and Tzeng, Shin-Cheng and Becker, Eric and Pazouki, Leila and Evans, Bradley and Cross, Fred and Cheng, Jianlin and Czymmek, Kirk and Schroda, Michael and Mühlhaus, Timo and Zhang, Ru</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">

</xml_diff>